<commit_message>
language features added and draft email language adjustments
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michalkassa/Desktop/lp-outreach/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3480E478-5B8E-B245-86E8-18E40A3D2BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09DB5B0D-C55A-934E-B546-40E303401B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="311">
   <si>
     <t>Country</t>
   </si>
@@ -212,9 +212,6 @@
     <t>vbv-vorsorgekasse-ag</t>
   </si>
   <si>
-    <t>&gt;€1.5B</t>
-  </si>
-  <si>
     <t>Confirmed private debt and stable real estate allocation despite capital guarantee structure</t>
   </si>
   <si>
@@ -293,9 +290,6 @@
     <t>nestle-pensionsfonds-ag</t>
   </si>
   <si>
-    <t>no contact</t>
-  </si>
-  <si>
     <t>integrated into German entity 2015 — do not contact</t>
   </si>
   <si>
@@ -945,13 +939,31 @@
   </si>
   <si>
     <t>Regulatory barrier or AUM too small</t>
+  </si>
+  <si>
+    <t>Christian Jacob</t>
+  </si>
+  <si>
+    <t>Chairman</t>
+  </si>
+  <si>
+    <t>NestleRente@neversa.de</t>
+  </si>
+  <si>
+    <t>€382.406M</t>
+  </si>
+  <si>
+    <t>€3.1717B</t>
+  </si>
+  <si>
+    <t>17.8B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -964,41 +976,56 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF375623"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF9C5700"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF833C00"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1068,10 +1095,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1079,26 +1107,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1106,17 +1122,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1492,7 +1512,7 @@
       <c r="D2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="15">
         <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1507,13 +1527,13 @@
       <c r="I2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="M2" s="2"/>
@@ -1532,7 +1552,7 @@
       <c r="D3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="15">
         <v>68</v>
       </c>
       <c r="F3" s="2" t="s">
@@ -1553,7 +1573,7 @@
       <c r="K3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="4" t="s">
         <v>32</v>
       </c>
       <c r="M3" s="2"/>
@@ -1572,7 +1592,7 @@
       <c r="D4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="15">
         <v>82</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -1593,7 +1613,7 @@
       <c r="K4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M4" s="2"/>
@@ -1612,7 +1632,7 @@
       <c r="D5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="15">
         <v>88</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -1633,7 +1653,7 @@
       <c r="K5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="4" t="s">
         <v>46</v>
       </c>
       <c r="M5" s="2"/>
@@ -1652,7 +1672,7 @@
       <c r="D6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="15">
         <v>78</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -1673,7 +1693,7 @@
       <c r="K6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="4" t="s">
         <v>53</v>
       </c>
       <c r="M6" s="2"/>
@@ -1692,28 +1712,20 @@
       <c r="D7" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="15">
         <v>25</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>56</v>
-      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="14"/>
       <c r="J7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="4" t="s">
         <v>57</v>
       </c>
       <c r="M7" s="2" t="s">
@@ -1734,11 +1746,11 @@
       <c r="D8" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="15">
         <v>58</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>62</v>
+        <v>310</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>19</v>
@@ -1755,53 +1767,53 @@
       <c r="K8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="L8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="M8" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="N8" s="2"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="15">
+        <v>5</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="9">
-        <v>5</v>
-      </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="K9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L9" s="7"/>
+      <c r="M9" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="K9" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="L9" s="11"/>
-      <c r="M9" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="N9" s="8"/>
+      <c r="N9" s="5"/>
     </row>
     <row r="10" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
@@ -1811,25 +1823,25 @@
         <v>15</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="15">
+        <v>48</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="12">
-        <v>48</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>31</v>
@@ -1837,8 +1849,8 @@
       <c r="K10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L10" s="5" t="s">
-        <v>79</v>
+      <c r="L10" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -1851,25 +1863,25 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="15">
+        <v>22</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="7">
-        <v>22</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>31</v>
@@ -1877,82 +1889,88 @@
       <c r="K11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L11" s="5"/>
+      <c r="L11" s="4"/>
       <c r="M11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="N11" s="2"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="8" t="s">
+      <c r="D12" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="15">
+        <v>5</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L12" s="7"/>
+      <c r="M12" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E12" s="9">
-        <v>5</v>
-      </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="L12" s="11"/>
-      <c r="M12" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="N12" s="8"/>
+      <c r="N12" s="5"/>
     </row>
     <row r="13" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="E13" s="15">
+        <v>50</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E13" s="12">
-        <v>50</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="J13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="L13" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -1965,25 +1983,25 @@
         <v>15</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" s="15">
+        <v>45</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E14" s="12">
-        <v>45</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>31</v>
@@ -1991,8 +2009,8 @@
       <c r="K14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L14" s="5" t="s">
-        <v>104</v>
+      <c r="L14" s="4" t="s">
+        <v>102</v>
       </c>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -2002,37 +2020,37 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="15">
+        <v>80</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="E15" s="3">
-        <v>80</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>110</v>
+        <v>95</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>108</v>
       </c>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -2042,37 +2060,37 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E16" s="15">
+        <v>68</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="E16" s="6">
-        <v>68</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>116</v>
+        <v>95</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
@@ -2082,40 +2100,40 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="15">
+        <v>48</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="E17" s="12">
-        <v>48</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I17" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L17" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="N17" s="2"/>
     </row>
@@ -2124,37 +2142,37 @@
         <v>14</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E18" s="12">
+        <v>123</v>
+      </c>
+      <c r="E18" s="15">
         <v>45</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L18" s="5" t="s">
-        <v>128</v>
+        <v>95</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>126</v>
       </c>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -2164,37 +2182,37 @@
         <v>14</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E19" s="15">
+        <v>80</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="E19" s="3">
-        <v>80</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>134</v>
+        <v>95</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>132</v>
       </c>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -2204,37 +2222,37 @@
         <v>14</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E20" s="12">
+        <v>134</v>
+      </c>
+      <c r="E20" s="15">
         <v>35</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L20" s="5" t="s">
-        <v>139</v>
+        <v>95</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -2244,40 +2262,40 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E21" s="15">
+        <v>32</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="E21" s="7">
-        <v>32</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I21" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L21" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="N21" s="2"/>
     </row>
@@ -2286,37 +2304,37 @@
         <v>14</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E22" s="15">
+        <v>55</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="E22" s="6">
-        <v>55</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>150</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>152</v>
+        <v>95</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>150</v>
       </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -2326,37 +2344,37 @@
         <v>14</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E23" s="15">
+        <v>62</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="E23" s="6">
-        <v>62</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L23" s="5" t="s">
-        <v>158</v>
+        <v>95</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -2366,99 +2384,99 @@
         <v>14</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="E24" s="12">
+        <v>158</v>
+      </c>
+      <c r="E24" s="15">
         <v>35</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L24" s="5" t="s">
-        <v>163</v>
+        <v>95</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>161</v>
       </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
     </row>
     <row r="25" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="E25" s="15">
+        <v>40</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="E25" s="12">
-        <v>40</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>170</v>
+        <v>95</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
     <row r="26" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E26" s="15">
+        <v>28</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E26" s="7">
-        <v>28</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>56</v>
@@ -2467,411 +2485,411 @@
         <v>29</v>
       </c>
       <c r="I26" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="N26" s="2"/>
     </row>
     <row r="27" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E27" s="15">
+        <v>28</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="E27" s="7">
-        <v>28</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I27" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L27" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="N27" s="2"/>
     </row>
     <row r="28" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="E28" s="7">
+        <v>183</v>
+      </c>
+      <c r="E28" s="15">
         <v>30</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>187</v>
+      <c r="I28" s="14" t="s">
+        <v>185</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L28" s="5" t="s">
-        <v>188</v>
+        <v>95</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>186</v>
       </c>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
     </row>
     <row r="29" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E29" s="12">
+        <v>188</v>
+      </c>
+      <c r="E29" s="15">
         <v>40</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L29" s="5" t="s">
-        <v>193</v>
+        <v>95</v>
+      </c>
+      <c r="L29" s="4" t="s">
+        <v>191</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
     <row r="30" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E30" s="12">
+        <v>193</v>
+      </c>
+      <c r="E30" s="15">
         <v>45</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L30" s="5" t="s">
-        <v>198</v>
+        <v>95</v>
+      </c>
+      <c r="L30" s="4" t="s">
+        <v>196</v>
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="E31" s="7">
+        <v>198</v>
+      </c>
+      <c r="E31" s="15">
         <v>30</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L31" s="5" t="s">
-        <v>203</v>
+        <v>95</v>
+      </c>
+      <c r="L31" s="4" t="s">
+        <v>201</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
     <row r="32" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E32" s="12">
+        <v>203</v>
+      </c>
+      <c r="E32" s="15">
         <v>38</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G32" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="J32" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L32" s="4" t="s">
         <v>207</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L32" s="5" t="s">
-        <v>209</v>
       </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
     <row r="33" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E33" s="15">
+        <v>25</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="E33" s="7">
-        <v>25</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L33" s="5" t="s">
-        <v>215</v>
+        <v>95</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>213</v>
       </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B34" s="8" t="s">
+      <c r="A34" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="E34" s="15">
+        <v>15</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="G34" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="E34" s="9">
+      <c r="H34" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L34" s="7"/>
+      <c r="M34" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="N34" s="5"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E35" s="15">
         <v>15</v>
       </c>
-      <c r="F34" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="J34" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K34" s="8" t="s">
+      <c r="F35" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K35" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="L34" s="11"/>
-      <c r="M34" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="N34" s="8"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A35" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="E35" s="9">
-        <v>15</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="H35" s="8" t="s">
+      <c r="L35" s="7"/>
+      <c r="M35" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="I35" s="8" t="s">
-        <v>228</v>
-      </c>
-      <c r="J35" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K35" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="L35" s="11"/>
-      <c r="M35" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="N35" s="8"/>
+      <c r="N35" s="5"/>
     </row>
     <row r="36" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="E36" s="15">
+        <v>22</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="E36" s="7">
-        <v>22</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>31</v>
@@ -2879,121 +2897,121 @@
       <c r="K36" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L36" s="5" t="s">
+      <c r="L36" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="N36" s="2"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="D37" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="N36" s="2"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A37" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="C37" s="8" t="s">
+      <c r="E37" s="15">
+        <v>15</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L37" s="7"/>
+      <c r="M37" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="N37" s="5"/>
+    </row>
+    <row r="38" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D38" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="E37" s="9">
-        <v>15</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="H37" s="8" t="s">
+      <c r="E38" s="15">
+        <v>18</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H38" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I37" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="J37" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K37" s="8" t="s">
+      <c r="I38" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K38" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="L37" s="11"/>
-      <c r="M37" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="N37" s="8"/>
-    </row>
-    <row r="38" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A38" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="E38" s="9">
-        <v>18</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="G38" s="8" t="s">
+      <c r="L38" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="H38" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="I38" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="J38" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="L38" s="11" t="s">
-        <v>244</v>
-      </c>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
     </row>
     <row r="39" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="E39" s="7">
+        <v>244</v>
+      </c>
+      <c r="E39" s="15">
         <v>20</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>31</v>
@@ -3001,41 +3019,41 @@
       <c r="K39" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L39" s="5" t="s">
-        <v>247</v>
+      <c r="L39" s="4" t="s">
+        <v>245</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="N39" s="2"/>
     </row>
     <row r="40" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E40" s="7">
+        <v>248</v>
+      </c>
+      <c r="E40" s="15">
         <v>22</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>31</v>
@@ -3043,81 +3061,81 @@
       <c r="K40" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L40" s="5" t="s">
+      <c r="L40" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="N40" s="2"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="M40" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="N40" s="2"/>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A41" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="C41" s="8" t="s">
+      <c r="E41" s="15">
+        <v>12</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="G41" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="H41" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I41" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="E41" s="9">
-        <v>12</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G41" s="8" t="s">
+      <c r="J41" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K41" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L41" s="7"/>
+      <c r="M41" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="H41" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="J41" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="K41" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="L41" s="11"/>
-      <c r="M41" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="N41" s="8"/>
+      <c r="N41" s="5"/>
     </row>
     <row r="42" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="E42" s="15">
+        <v>52</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="G42" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="E42" s="12">
-        <v>52</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>262</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>31</v>
@@ -3125,39 +3143,39 @@
       <c r="K42" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L42" s="5" t="s">
-        <v>264</v>
+      <c r="L42" s="4" t="s">
+        <v>262</v>
       </c>
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
     <row r="43" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E43" s="15">
+        <v>42</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="G43" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="E43" s="12">
-        <v>42</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>268</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>31</v>
@@ -3165,39 +3183,39 @@
       <c r="K43" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L43" s="5" t="s">
-        <v>270</v>
+      <c r="L43" s="4" t="s">
+        <v>268</v>
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
     <row r="44" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E44" s="15">
+        <v>80</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="G44" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="E44" s="3">
-        <v>80</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>274</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>31</v>
@@ -3205,39 +3223,39 @@
       <c r="K44" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L44" s="5" t="s">
-        <v>276</v>
+      <c r="L44" s="4" t="s">
+        <v>274</v>
       </c>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
     </row>
     <row r="45" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E45" s="15">
+        <v>50</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="E45" s="12">
-        <v>50</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>31</v>
@@ -3245,39 +3263,39 @@
       <c r="K45" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L45" s="5" t="s">
-        <v>282</v>
+      <c r="L45" s="4" t="s">
+        <v>280</v>
       </c>
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
     <row r="46" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E46" s="15">
+        <v>72</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="E46" s="6">
-        <v>72</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>286</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>31</v>
@@ -3285,14 +3303,18 @@
       <c r="K46" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L46" s="5" t="s">
-        <v>288</v>
+      <c r="L46" s="4" t="s">
+        <v>286</v>
       </c>
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="I12" r:id="rId1" xr:uid="{5175B0FD-4849-1A41-AE4B-FCD228965C29}"/>
+    <hyperlink ref="I28" r:id="rId2" xr:uid="{265E74FE-C55A-3A48-A85D-71032C12D1BE}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3309,69 +3331,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="B1" s="13" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="B2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="C2" t="s">
         <v>292</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="C3" t="s">
         <v>295</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="16" t="s">
+      <c r="C4" t="s">
         <v>298</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
         <v>299</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="17" t="s">
+      <c r="C5" t="s">
         <v>301</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="C6" t="s">
         <v>304</v>
-      </c>
-      <c r="B6" t="s">
-        <v>305</v>
-      </c>
-      <c r="C6" t="s">
-        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>